<commit_message>
new changes final project
</commit_message>
<xml_diff>
--- a/miranda_bonus_chartQ13.xlsx
+++ b/miranda_bonus_chartQ13.xlsx
@@ -8,23 +8,24 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nataliamiranda\Documents\DATA_Labs\Capstone_1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8BE270E-216E-4D7D-83EF-8F505EF24C2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21537869-F2F5-40F9-B5BE-8C3B27A13468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{83F94563-6C32-4839-B94A-179D20B041ED}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{83F94563-6C32-4839-B94A-179D20B041ED}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
-    <sheet name="miranda_bonus_chartQ13" sheetId="1" r:id="rId2"/>
+    <sheet name="Detail1" sheetId="3" r:id="rId1"/>
+    <sheet name="PIVOTCHART" sheetId="2" r:id="rId2"/>
+    <sheet name="miranda_bonus_chartQ13" sheetId="1" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId3"/>
+    <pivotCache cacheId="0" r:id="rId4"/>
   </pivotCaches>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="33">
   <si>
     <t>SalesManager</t>
   </si>
@@ -120,6 +121,9 @@
   </si>
   <si>
     <t>Row Labels</t>
+  </si>
+  <si>
+    <t>Details for Sum of TotalRevenue</t>
   </si>
 </sst>
 </file>
@@ -603,7 +607,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -612,6 +616,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" indent="1"/>
     </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -684,7 +689,7 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[miranda_bonus_chartQ13.xlsx]Sheet1!PivotTable1</c:name>
+    <c:name>[miranda_bonus_chartQ13.xlsx]PIVOTCHART!PivotTable1</c:name>
     <c:fmtId val="0"/>
   </c:pivotSource>
   <c:chart>
@@ -1637,7 +1642,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$B$1:$B$2</c:f>
+              <c:f>PIVOTCHART!$B$1:$B$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1715,7 +1720,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -1769,7 +1774,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$B$3:$B$17</c:f>
+              <c:f>PIVOTCHART!$B$3:$B$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1790,7 +1795,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$C$1:$C$2</c:f>
+              <c:f>PIVOTCHART!$C$1:$C$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1868,7 +1873,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -1922,7 +1927,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$C$3:$C$17</c:f>
+              <c:f>PIVOTCHART!$C$3:$C$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -1943,7 +1948,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$D$1:$D$2</c:f>
+              <c:f>PIVOTCHART!$D$1:$D$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2021,7 +2026,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2075,7 +2080,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$D$3:$D$17</c:f>
+              <c:f>PIVOTCHART!$D$3:$D$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2096,7 +2101,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$E$1:$E$2</c:f>
+              <c:f>PIVOTCHART!$E$1:$E$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2174,7 +2179,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2228,7 +2233,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$E$3:$E$17</c:f>
+              <c:f>PIVOTCHART!$E$3:$E$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2249,7 +2254,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$F$1:$F$2</c:f>
+              <c:f>PIVOTCHART!$F$1:$F$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2327,7 +2332,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2381,7 +2386,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$3:$F$17</c:f>
+              <c:f>PIVOTCHART!$F$3:$F$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2402,7 +2407,7 @@
           <c:order val="5"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$G$1:$G$2</c:f>
+              <c:f>PIVOTCHART!$G$1:$G$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2480,7 +2485,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2534,7 +2539,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$G$3:$G$17</c:f>
+              <c:f>PIVOTCHART!$G$3:$G$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2555,7 +2560,7 @@
           <c:order val="6"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$H$1:$H$2</c:f>
+              <c:f>PIVOTCHART!$H$1:$H$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2635,7 +2640,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2689,7 +2694,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$H$3:$H$17</c:f>
+              <c:f>PIVOTCHART!$H$3:$H$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2710,7 +2715,7 @@
           <c:order val="7"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$I$1:$I$2</c:f>
+              <c:f>PIVOTCHART!$I$1:$I$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2790,7 +2795,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2844,7 +2849,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$I$3:$I$17</c:f>
+              <c:f>PIVOTCHART!$I$3:$I$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -2865,7 +2870,7 @@
           <c:order val="8"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$J$1:$J$2</c:f>
+              <c:f>PIVOTCHART!$J$1:$J$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -2945,7 +2950,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -2999,7 +3004,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$J$3:$J$17</c:f>
+              <c:f>PIVOTCHART!$J$3:$J$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -3020,7 +3025,7 @@
           <c:order val="9"/>
           <c:tx>
             <c:strRef>
-              <c:f>Sheet1!$K$1:$K$2</c:f>
+              <c:f>PIVOTCHART!$K$1:$K$2</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3100,7 +3105,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Sheet1!$A$3:$A$17</c:f>
+              <c:f>PIVOTCHART!$A$3:$A$17</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="10"/>
                 <c:lvl>
@@ -3154,7 +3159,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$K$3:$K$17</c:f>
+              <c:f>PIVOTCHART!$K$3:$K$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="10"/>
@@ -4475,6 +4480,19 @@
 </pivotTableDefinition>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4D900F2E-27E9-4996-B636-5E55B85CA186}" name="Table1" displayName="Table1" ref="A3:D13" totalsRowShown="0">
+  <autoFilter ref="A3:D13" xr:uid="{4D900F2E-27E9-4996-B636-5E55B85CA186}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{5A0A167F-5F29-4359-B297-D40A9EEECC88}" name="SalesManager"/>
+    <tableColumn id="2" xr3:uid="{F3C993F0-9305-40E6-9B29-26ADB25DE763}" name="State"/>
+    <tableColumn id="3" xr3:uid="{8E1EC976-68C8-4FB7-BBFE-FCE95D6F0561}" name="Region"/>
+    <tableColumn id="4" xr3:uid="{8EC9F2E6-59F2-4189-A229-11821E0DCAD5}" name="TotalRevenue"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -4791,6 +4809,184 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D660726A-9448-4169-83A9-86A754D7FB76}">
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="18.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.453125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A1" s="4" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>6</v>
+      </c>
+      <c r="D4">
+        <v>5733256.2699999996</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B5" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5">
+        <v>2392222.44</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" t="s">
+        <v>25</v>
+      </c>
+      <c r="C6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D6">
+        <v>1877249.75</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7">
+        <v>3417850.01</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" t="s">
+        <v>9</v>
+      </c>
+      <c r="D8">
+        <v>6412632.2199999997</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B9" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9">
+        <v>3930187.55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A10" t="s">
+        <v>26</v>
+      </c>
+      <c r="B10" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10">
+        <v>648812.56000000006</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A11" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>6</v>
+      </c>
+      <c r="D11">
+        <v>5175405.87</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" t="s">
+        <v>15</v>
+      </c>
+      <c r="C12" t="s">
+        <v>16</v>
+      </c>
+      <c r="D12">
+        <v>4330817.09</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A13" t="s">
+        <v>4</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13">
+        <v>11451615.09</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{678FDE8B-9904-4A1B-85C6-5050F29CDE29}">
   <dimension ref="A1:L17"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
@@ -5079,7 +5275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{499DDB63-0A66-43A3-8550-5881E938F726}">
   <dimension ref="A1:D11"/>
   <sheetFormatPr defaultColWidth="18.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>

</xml_diff>